<commit_message>
Atualizacao de arquivos - 01/10/2026 10:11:02,57
</commit_message>
<xml_diff>
--- a/backlog_churn.xlsx
+++ b/backlog_churn.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="29">
   <si>
     <t>Mês</t>
   </si>
@@ -67,6 +67,9 @@
     <t>December</t>
   </si>
   <si>
+    <t>Setembro</t>
+  </si>
+  <si>
     <t>House Hold</t>
   </si>
   <si>
@@ -76,6 +79,15 @@
     <t>Large Corporate</t>
   </si>
   <si>
+    <t>Corporativo</t>
+  </si>
+  <si>
+    <t>PF</t>
+  </si>
+  <si>
+    <t>PME</t>
+  </si>
+  <si>
     <t>Voluntary Churn</t>
   </si>
   <si>
@@ -83,6 +95,12 @@
   </si>
   <si>
     <t>Adjustments</t>
+  </si>
+  <si>
+    <t>Involuntário</t>
+  </si>
+  <si>
+    <t>Voluntário</t>
   </si>
 </sst>
 </file>
@@ -414,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E182"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -445,10 +463,10 @@
         <v>603</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -462,10 +480,10 @@
         <v>152</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -479,10 +497,10 @@
         <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -496,10 +514,10 @@
         <v>613</v>
       </c>
       <c r="D5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -513,10 +531,10 @@
         <v>224</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -530,10 +548,10 @@
         <v>29</v>
       </c>
       <c r="D7" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -547,10 +565,10 @@
         <v>0</v>
       </c>
       <c r="D8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -564,10 +582,10 @@
         <v>0</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -581,10 +599,10 @@
         <v>0</v>
       </c>
       <c r="D10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -598,10 +616,10 @@
         <v>649</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -615,10 +633,10 @@
         <v>197</v>
       </c>
       <c r="D12" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -632,10 +650,10 @@
         <v>105</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -649,10 +667,10 @@
         <v>613</v>
       </c>
       <c r="D14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -666,10 +684,10 @@
         <v>188</v>
       </c>
       <c r="D15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -683,10 +701,10 @@
         <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -700,10 +718,10 @@
         <v>0</v>
       </c>
       <c r="D17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E17" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -717,10 +735,10 @@
         <v>0</v>
       </c>
       <c r="D18" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E18" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -734,10 +752,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -751,10 +769,10 @@
         <v>759</v>
       </c>
       <c r="D20" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -768,10 +786,10 @@
         <v>253</v>
       </c>
       <c r="D21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -785,10 +803,10 @@
         <v>116</v>
       </c>
       <c r="D22" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -802,10 +820,10 @@
         <v>486</v>
       </c>
       <c r="D23" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E23" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -819,10 +837,10 @@
         <v>135</v>
       </c>
       <c r="D24" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E24" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -836,10 +854,10 @@
         <v>9</v>
       </c>
       <c r="D25" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -853,10 +871,10 @@
         <v>0</v>
       </c>
       <c r="D26" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E26" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -870,10 +888,10 @@
         <v>0</v>
       </c>
       <c r="D27" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E27" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -887,10 +905,10 @@
         <v>0</v>
       </c>
       <c r="D28" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -904,10 +922,10 @@
         <v>658</v>
       </c>
       <c r="D29" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E29" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -921,10 +939,10 @@
         <v>206</v>
       </c>
       <c r="D30" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E30" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -938,10 +956,10 @@
         <v>107</v>
       </c>
       <c r="D31" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E31" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -955,10 +973,10 @@
         <v>663</v>
       </c>
       <c r="D32" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E32" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -972,10 +990,10 @@
         <v>197</v>
       </c>
       <c r="D33" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E33" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -989,10 +1007,10 @@
         <v>9</v>
       </c>
       <c r="D34" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E34" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1006,10 +1024,10 @@
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E35" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1023,10 +1041,10 @@
         <v>0</v>
       </c>
       <c r="D36" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E36" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1040,10 +1058,10 @@
         <v>0</v>
       </c>
       <c r="D37" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E37" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1057,10 +1075,10 @@
         <v>611</v>
       </c>
       <c r="D38" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E38" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -1074,10 +1092,10 @@
         <v>220</v>
       </c>
       <c r="D39" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E39" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1091,10 +1109,10 @@
         <v>375</v>
       </c>
       <c r="D40" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E40" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1108,10 +1126,10 @@
         <v>893</v>
       </c>
       <c r="D41" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E41" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -1125,10 +1143,10 @@
         <v>244</v>
       </c>
       <c r="D42" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E42" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -1142,10 +1160,10 @@
         <v>4</v>
       </c>
       <c r="D43" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E43" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -1159,10 +1177,10 @@
         <v>0</v>
       </c>
       <c r="D44" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E44" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -1176,10 +1194,10 @@
         <v>0</v>
       </c>
       <c r="D45" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E45" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -1193,10 +1211,10 @@
         <v>0</v>
       </c>
       <c r="D46" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E46" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -1210,10 +1228,10 @@
         <v>671</v>
       </c>
       <c r="D47" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E47" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -1227,10 +1245,10 @@
         <v>221</v>
       </c>
       <c r="D48" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E48" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -1244,10 +1262,10 @@
         <v>263</v>
       </c>
       <c r="D49" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E49" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -1261,10 +1279,10 @@
         <v>974</v>
       </c>
       <c r="D50" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E50" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -1278,10 +1296,10 @@
         <v>281</v>
       </c>
       <c r="D51" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E51" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -1295,10 +1313,10 @@
         <v>7</v>
       </c>
       <c r="D52" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E52" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -1312,10 +1330,10 @@
         <v>0</v>
       </c>
       <c r="D53" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E53" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -1329,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="D54" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E54" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -1346,10 +1364,10 @@
         <v>0</v>
       </c>
       <c r="D55" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E55" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -1363,10 +1381,10 @@
         <v>883</v>
       </c>
       <c r="D56" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E56" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -1380,10 +1398,10 @@
         <v>243</v>
       </c>
       <c r="D57" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E57" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -1397,10 +1415,10 @@
         <v>127</v>
       </c>
       <c r="D58" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E58" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -1414,10 +1432,10 @@
         <v>983</v>
       </c>
       <c r="D59" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E59" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -1431,10 +1449,10 @@
         <v>307</v>
       </c>
       <c r="D60" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E60" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -1448,10 +1466,10 @@
         <v>9</v>
       </c>
       <c r="D61" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E61" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="62" spans="1:5">
@@ -1465,10 +1483,10 @@
         <v>0</v>
       </c>
       <c r="D62" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E62" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="63" spans="1:5">
@@ -1482,10 +1500,10 @@
         <v>0</v>
       </c>
       <c r="D63" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E63" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="64" spans="1:5">
@@ -1499,10 +1517,10 @@
         <v>0</v>
       </c>
       <c r="D64" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E64" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="65" spans="1:5">
@@ -1516,10 +1534,10 @@
         <v>867</v>
       </c>
       <c r="D65" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E65" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="66" spans="1:5">
@@ -1533,10 +1551,10 @@
         <v>267</v>
       </c>
       <c r="D66" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E66" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="67" spans="1:5">
@@ -1550,10 +1568,10 @@
         <v>161</v>
       </c>
       <c r="D67" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E67" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="68" spans="1:5">
@@ -1567,10 +1585,10 @@
         <v>795</v>
       </c>
       <c r="D68" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E68" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -1584,10 +1602,10 @@
         <v>257</v>
       </c>
       <c r="D69" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E69" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -1601,10 +1619,10 @@
         <v>10</v>
       </c>
       <c r="D70" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E70" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -1618,10 +1636,10 @@
         <v>0</v>
       </c>
       <c r="D71" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E71" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="72" spans="1:5">
@@ -1635,10 +1653,10 @@
         <v>0</v>
       </c>
       <c r="D72" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E72" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="73" spans="1:5">
@@ -1652,10 +1670,10 @@
         <v>0</v>
       </c>
       <c r="D73" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E73" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="74" spans="1:5">
@@ -1669,10 +1687,10 @@
         <v>842</v>
       </c>
       <c r="D74" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E74" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="75" spans="1:5">
@@ -1686,10 +1704,10 @@
         <v>251</v>
       </c>
       <c r="D75" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E75" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="76" spans="1:5">
@@ -1703,10 +1721,10 @@
         <v>172</v>
       </c>
       <c r="D76" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E76" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77" spans="1:5">
@@ -1720,10 +1738,10 @@
         <v>672</v>
       </c>
       <c r="D77" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E77" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="78" spans="1:5">
@@ -1737,10 +1755,10 @@
         <v>198</v>
       </c>
       <c r="D78" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E78" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="79" spans="1:5">
@@ -1754,10 +1772,10 @@
         <v>8</v>
       </c>
       <c r="D79" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E79" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="80" spans="1:5">
@@ -1771,10 +1789,10 @@
         <v>0</v>
       </c>
       <c r="D80" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E80" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="81" spans="1:5">
@@ -1788,10 +1806,10 @@
         <v>0</v>
       </c>
       <c r="D81" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E81" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="82" spans="1:5">
@@ -1805,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="D82" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E82" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="83" spans="1:5">
@@ -1822,10 +1840,10 @@
         <v>829</v>
       </c>
       <c r="D83" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E83" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="84" spans="1:5">
@@ -1839,10 +1857,10 @@
         <v>256</v>
       </c>
       <c r="D84" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E84" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="85" spans="1:5">
@@ -1856,10 +1874,10 @@
         <v>114</v>
       </c>
       <c r="D85" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E85" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -1873,10 +1891,10 @@
         <v>820</v>
       </c>
       <c r="D86" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E86" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="87" spans="1:5">
@@ -1890,10 +1908,10 @@
         <v>212</v>
       </c>
       <c r="D87" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E87" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="88" spans="1:5">
@@ -1907,10 +1925,10 @@
         <v>4</v>
       </c>
       <c r="D88" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E88" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="89" spans="1:5">
@@ -1924,10 +1942,10 @@
         <v>0</v>
       </c>
       <c r="D89" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E89" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="90" spans="1:5">
@@ -1941,10 +1959,10 @@
         <v>0</v>
       </c>
       <c r="D90" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E90" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="91" spans="1:5">
@@ -1958,10 +1976,10 @@
         <v>0</v>
       </c>
       <c r="D91" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E91" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="92" spans="1:5">
@@ -1975,10 +1993,10 @@
         <v>1026</v>
       </c>
       <c r="D92" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E92" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="93" spans="1:5">
@@ -1992,10 +2010,10 @@
         <v>312</v>
       </c>
       <c r="D93" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E93" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="94" spans="1:5">
@@ -2009,10 +2027,10 @@
         <v>116</v>
       </c>
       <c r="D94" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E94" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="95" spans="1:5">
@@ -2026,10 +2044,10 @@
         <v>787</v>
       </c>
       <c r="D95" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E95" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="96" spans="1:5">
@@ -2043,10 +2061,10 @@
         <v>252</v>
       </c>
       <c r="D96" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E96" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="97" spans="1:5">
@@ -2060,10 +2078,10 @@
         <v>3</v>
       </c>
       <c r="D97" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E97" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="98" spans="1:5">
@@ -2077,10 +2095,10 @@
         <v>0</v>
       </c>
       <c r="D98" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E98" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="99" spans="1:5">
@@ -2094,10 +2112,10 @@
         <v>0</v>
       </c>
       <c r="D99" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E99" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="100" spans="1:5">
@@ -2111,10 +2129,10 @@
         <v>0</v>
       </c>
       <c r="D100" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E100" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="101" spans="1:5">
@@ -2128,10 +2146,10 @@
         <v>1026</v>
       </c>
       <c r="D101" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E101" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="102" spans="1:5">
@@ -2145,10 +2163,10 @@
         <v>312</v>
       </c>
       <c r="D102" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E102" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="103" spans="1:5">
@@ -2162,10 +2180,10 @@
         <v>116</v>
       </c>
       <c r="D103" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E103" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="104" spans="1:5">
@@ -2179,10 +2197,10 @@
         <v>787</v>
       </c>
       <c r="D104" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E104" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="105" spans="1:5">
@@ -2196,10 +2214,10 @@
         <v>252</v>
       </c>
       <c r="D105" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E105" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="106" spans="1:5">
@@ -2213,10 +2231,10 @@
         <v>3</v>
       </c>
       <c r="D106" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E106" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="107" spans="1:5">
@@ -2230,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="D107" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E107" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="108" spans="1:5">
@@ -2247,10 +2265,10 @@
         <v>0</v>
       </c>
       <c r="D108" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E108" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="109" spans="1:5">
@@ -2264,10 +2282,10 @@
         <v>0</v>
       </c>
       <c r="D109" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E109" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="110" spans="1:5">
@@ -2281,10 +2299,10 @@
         <v>1213</v>
       </c>
       <c r="D110" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E110" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="111" spans="1:5">
@@ -2298,10 +2316,10 @@
         <v>385</v>
       </c>
       <c r="D111" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E111" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2315,10 +2333,10 @@
         <v>114</v>
       </c>
       <c r="D112" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E112" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="113" spans="1:5">
@@ -2332,10 +2350,10 @@
         <v>766</v>
       </c>
       <c r="D113" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E113" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="114" spans="1:5">
@@ -2349,10 +2367,10 @@
         <v>284</v>
       </c>
       <c r="D114" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E114" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="115" spans="1:5">
@@ -2366,10 +2384,10 @@
         <v>21</v>
       </c>
       <c r="D115" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E115" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="116" spans="1:5">
@@ -2383,10 +2401,10 @@
         <v>0</v>
       </c>
       <c r="D116" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E116" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="117" spans="1:5">
@@ -2400,10 +2418,10 @@
         <v>0</v>
       </c>
       <c r="D117" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E117" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="118" spans="1:5">
@@ -2417,10 +2435,10 @@
         <v>0</v>
       </c>
       <c r="D118" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E118" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="119" spans="1:5">
@@ -2434,10 +2452,10 @@
         <v>1342</v>
       </c>
       <c r="D119" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E119" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="120" spans="1:5">
@@ -2451,10 +2469,10 @@
         <v>398</v>
       </c>
       <c r="D120" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E120" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="121" spans="1:5">
@@ -2468,10 +2486,10 @@
         <v>246</v>
       </c>
       <c r="D121" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E121" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="122" spans="1:5">
@@ -2485,10 +2503,10 @@
         <v>719</v>
       </c>
       <c r="D122" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E122" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="123" spans="1:5">
@@ -2502,10 +2520,10 @@
         <v>103</v>
       </c>
       <c r="D123" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E123" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="124" spans="1:5">
@@ -2519,10 +2537,10 @@
         <v>99</v>
       </c>
       <c r="D124" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E124" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125" spans="1:5">
@@ -2536,10 +2554,10 @@
         <v>0</v>
       </c>
       <c r="D125" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E125" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="126" spans="1:5">
@@ -2553,10 +2571,10 @@
         <v>0</v>
       </c>
       <c r="D126" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E126" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="127" spans="1:5">
@@ -2570,10 +2588,10 @@
         <v>0</v>
       </c>
       <c r="D127" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E127" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="128" spans="1:5">
@@ -2587,10 +2605,10 @@
         <v>1446</v>
       </c>
       <c r="D128" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E128" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="129" spans="1:5">
@@ -2604,10 +2622,10 @@
         <v>506</v>
       </c>
       <c r="D129" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E129" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="130" spans="1:5">
@@ -2621,10 +2639,10 @@
         <v>147</v>
       </c>
       <c r="D130" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E130" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="131" spans="1:5">
@@ -2638,10 +2656,10 @@
         <v>618</v>
       </c>
       <c r="D131" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E131" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="132" spans="1:5">
@@ -2655,10 +2673,10 @@
         <v>109</v>
       </c>
       <c r="D132" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E132" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="133" spans="1:5">
@@ -2672,10 +2690,10 @@
         <v>46</v>
       </c>
       <c r="D133" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E133" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="134" spans="1:5">
@@ -2689,10 +2707,10 @@
         <v>0</v>
       </c>
       <c r="D134" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E134" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="135" spans="1:5">
@@ -2706,10 +2724,10 @@
         <v>0</v>
       </c>
       <c r="D135" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E135" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="136" spans="1:5">
@@ -2723,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="D136" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E136" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="137" spans="1:5">
@@ -2740,10 +2758,10 @@
         <v>1400</v>
       </c>
       <c r="D137" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E137" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="138" spans="1:5">
@@ -2757,10 +2775,10 @@
         <v>441</v>
       </c>
       <c r="D138" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E138" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="139" spans="1:5">
@@ -2774,10 +2792,10 @@
         <v>228</v>
       </c>
       <c r="D139" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E139" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="140" spans="1:5">
@@ -2791,10 +2809,10 @@
         <v>488</v>
       </c>
       <c r="D140" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E140" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="141" spans="1:5">
@@ -2808,10 +2826,10 @@
         <v>245</v>
       </c>
       <c r="D141" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E141" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="142" spans="1:5">
@@ -2825,10 +2843,10 @@
         <v>24</v>
       </c>
       <c r="D142" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E142" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="143" spans="1:5">
@@ -2842,10 +2860,10 @@
         <v>0</v>
       </c>
       <c r="D143" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E143" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="144" spans="1:5">
@@ -2859,10 +2877,10 @@
         <v>0</v>
       </c>
       <c r="D144" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E144" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="145" spans="1:5">
@@ -2876,10 +2894,10 @@
         <v>0</v>
       </c>
       <c r="D145" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E145" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="146" spans="1:5">
@@ -2893,10 +2911,10 @@
         <v>1337</v>
       </c>
       <c r="D146" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E146" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="147" spans="1:5">
@@ -2910,10 +2928,10 @@
         <v>421</v>
       </c>
       <c r="D147" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E147" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="148" spans="1:5">
@@ -2927,10 +2945,10 @@
         <v>220</v>
       </c>
       <c r="D148" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E148" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="149" spans="1:5">
@@ -2944,10 +2962,10 @@
         <v>311</v>
       </c>
       <c r="D149" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E149" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="150" spans="1:5">
@@ -2961,10 +2979,10 @@
         <v>169</v>
       </c>
       <c r="D150" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E150" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="151" spans="1:5">
@@ -2978,10 +2996,10 @@
         <v>24</v>
       </c>
       <c r="D151" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E151" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="152" spans="1:5">
@@ -2995,10 +3013,10 @@
         <v>0</v>
       </c>
       <c r="D152" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E152" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="153" spans="1:5">
@@ -3012,10 +3030,10 @@
         <v>0</v>
       </c>
       <c r="D153" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E153" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="154" spans="1:5">
@@ -3029,10 +3047,10 @@
         <v>0</v>
       </c>
       <c r="D154" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E154" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="155" spans="1:5">
@@ -3046,10 +3064,10 @@
         <v>602</v>
       </c>
       <c r="D155" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E155" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="156" spans="1:5">
@@ -3063,10 +3081,10 @@
         <v>1635</v>
       </c>
       <c r="D156" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E156" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="157" spans="1:5">
@@ -3080,10 +3098,10 @@
         <v>4</v>
       </c>
       <c r="D157" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E157" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="158" spans="1:5">
@@ -3097,10 +3115,10 @@
         <v>244</v>
       </c>
       <c r="D158" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E158" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="159" spans="1:5">
@@ -3114,10 +3132,10 @@
         <v>99</v>
       </c>
       <c r="D159" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E159" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="160" spans="1:5">
@@ -3131,10 +3149,10 @@
         <v>847</v>
       </c>
       <c r="D160" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E160" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="161" spans="1:5">
@@ -3148,10 +3166,10 @@
         <v>1472</v>
       </c>
       <c r="D161" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E161" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="162" spans="1:5">
@@ -3165,10 +3183,10 @@
         <v>1</v>
       </c>
       <c r="D162" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E162" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="163" spans="1:5">
@@ -3182,10 +3200,10 @@
         <v>246</v>
       </c>
       <c r="D163" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E163" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="164" spans="1:5">
@@ -3199,10 +3217,10 @@
         <v>2</v>
       </c>
       <c r="D164" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E164" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="165" spans="1:5">
@@ -3216,10 +3234,10 @@
         <v>115</v>
       </c>
       <c r="D165" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E165" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="166" spans="1:5">
@@ -3233,10 +3251,10 @@
         <v>807</v>
       </c>
       <c r="D166" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E166" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="167" spans="1:5">
@@ -3250,10 +3268,10 @@
         <v>1465</v>
       </c>
       <c r="D167" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E167" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="168" spans="1:5">
@@ -3267,10 +3285,10 @@
         <v>1</v>
       </c>
       <c r="D168" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E168" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="169" spans="1:5">
@@ -3284,10 +3302,10 @@
         <v>247</v>
       </c>
       <c r="D169" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E169" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="170" spans="1:5">
@@ -3301,10 +3319,10 @@
         <v>2</v>
       </c>
       <c r="D170" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E170" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="171" spans="1:5">
@@ -3318,10 +3336,197 @@
         <v>114</v>
       </c>
       <c r="D171" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E171" t="s">
-        <v>20</v>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5">
+      <c r="A172" t="s">
+        <v>17</v>
+      </c>
+      <c r="B172">
+        <v>2026</v>
+      </c>
+      <c r="C172">
+        <v>3</v>
+      </c>
+      <c r="D172" t="s">
+        <v>21</v>
+      </c>
+      <c r="E172" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5">
+      <c r="A173" t="s">
+        <v>17</v>
+      </c>
+      <c r="B173">
+        <v>2026</v>
+      </c>
+      <c r="C173">
+        <v>456</v>
+      </c>
+      <c r="D173" t="s">
+        <v>21</v>
+      </c>
+      <c r="E173" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5">
+      <c r="A174" t="s">
+        <v>17</v>
+      </c>
+      <c r="B174">
+        <v>2026</v>
+      </c>
+      <c r="C174">
+        <v>1047</v>
+      </c>
+      <c r="D174" t="s">
+        <v>22</v>
+      </c>
+      <c r="E174" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5">
+      <c r="A175" t="s">
+        <v>17</v>
+      </c>
+      <c r="B175">
+        <v>2026</v>
+      </c>
+      <c r="C175">
+        <v>1034</v>
+      </c>
+      <c r="D175" t="s">
+        <v>22</v>
+      </c>
+      <c r="E175" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5">
+      <c r="A176" t="s">
+        <v>17</v>
+      </c>
+      <c r="B176">
+        <v>2026</v>
+      </c>
+      <c r="C176">
+        <v>4</v>
+      </c>
+      <c r="D176" t="s">
+        <v>23</v>
+      </c>
+      <c r="E176" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5">
+      <c r="A177" t="s">
+        <v>17</v>
+      </c>
+      <c r="B177">
+        <v>2026</v>
+      </c>
+      <c r="C177">
+        <v>275</v>
+      </c>
+      <c r="D177" t="s">
+        <v>23</v>
+      </c>
+      <c r="E177" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5">
+      <c r="A178" t="s">
+        <v>14</v>
+      </c>
+      <c r="B178">
+        <v>2026</v>
+      </c>
+      <c r="C178">
+        <v>1192</v>
+      </c>
+      <c r="D178" t="s">
+        <v>18</v>
+      </c>
+      <c r="E178" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5">
+      <c r="A179" t="s">
+        <v>14</v>
+      </c>
+      <c r="B179">
+        <v>2026</v>
+      </c>
+      <c r="C179">
+        <v>1288</v>
+      </c>
+      <c r="D179" t="s">
+        <v>18</v>
+      </c>
+      <c r="E179" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5">
+      <c r="A180" t="s">
+        <v>14</v>
+      </c>
+      <c r="B180">
+        <v>2026</v>
+      </c>
+      <c r="C180">
+        <v>257</v>
+      </c>
+      <c r="D180" t="s">
+        <v>20</v>
+      </c>
+      <c r="E180" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5">
+      <c r="A181" t="s">
+        <v>14</v>
+      </c>
+      <c r="B181">
+        <v>2026</v>
+      </c>
+      <c r="C181">
+        <v>2</v>
+      </c>
+      <c r="D181" t="s">
+        <v>19</v>
+      </c>
+      <c r="E181" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5">
+      <c r="A182" t="s">
+        <v>14</v>
+      </c>
+      <c r="B182">
+        <v>2026</v>
+      </c>
+      <c r="C182">
+        <v>91</v>
+      </c>
+      <c r="D182" t="s">
+        <v>19</v>
+      </c>
+      <c r="E182" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>